<commit_message>
baselines: unify the 5 shared held-out reports on the regenerated ruler
Qualys/Nessus scan-b and the 3 held-out ZAPs existed in two near-identical
derivations (original converter + trim vs regenerated from the export +
trim). Keep the regenerated one everywhere: reproducible from the raw export
by make_heldout_baselines.py, and a single provenance chain shared with the
training gold. Verified field-equal (normalized) to the originals before the
switch.
</commit_message>
<xml_diff>
--- a/resources/zap/ZAP_JBoss7.xlsx
+++ b/resources/zap/ZAP_JBoss7.xlsx
@@ -486,12 +486,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Content Security Policy (CSP) is an added layer of security that helps to detect and mitigate certain types of attacks, including Cross Site Scripting (XSS) and data injection attacks. These attacks are used for everything from data theft to site defacement or distribution of malware. CSP provides a set of standard HTTP headers that allow website owners to declare approved sources of content that browsers should be allowed to load on that page — covered types are JavaScript, CSS, HTML frames, fonts, images and embeddable objects such as Java applets, ActiveX, audio and video files.</t>
+          <t>['Content Security Policy (CSP) is an added layer of security that helps to detect and mitigate certain types of attacks, including Cross Site Scripting (XSS) and data injection attacks. These attacks are used for everything from data theft to site defacement or distribution of malware. CSP provides a set of standard HTTP headers that allow website owners to declare approved sources of content that browsers should be allowed to load on that page — covered types are JavaScript, CSS, HTML frames, fonts, images and embeddable objects such as Java applets, ActiveX, audio and video files.']</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ensure that your web server, application server, load balancer, etc. is configured to set the Content-Security-Policy header.</t>
+          <t>['Ensure that your web server, application server, load balancer, etc. is configured to set the Content-Security-Policy header.']</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -530,13 +530,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The response does not protect against 'ClickJacking' attacks. It should include either Content-Security-Policy with 'frame-ancestors' directive or X-Frame-Options.</t>
+          <t>["The response does not protect against 'ClickJacking' attacks. It should include either Content-Security-Policy with 'frame-ancestors' directive or X-Frame-Options."]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Modern Web browsers support the Content-Security-Policy and X-Frame-Options HTTP headers. Ensure one of them is set on all web pages returned by your site/app.
-If you expect the page to be framed only by pages on your server (e.g. it's part of a FRAMESET) then you'll want to use SAMEORIGIN, otherwise if you never expect the page to be framed, you should use DENY. Alternatively consider implementing Content Security Policy's "frame-ancestors" directive.</t>
+          <t>['Modern Web browsers support the Content-Security-Policy and X-Frame-Options HTTP headers. Ensure one of them is set on all web pages returned by your site/app.', 'If you expect the page to be framed only by pages on your server (e.g. it\'s part of a FRAMESET) then you\'ll want to use SAMEORIGIN, otherwise if you never expect the page to be framed, you should use DENY. Alternatively consider implementing Content Security Policy\'s "frame-ancestors" directive.']</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -575,12 +574,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>The web/application server is leaking information via one or more "X-Powered-By" HTTP response headers. Access to such information may facilitate attackers identifying other frameworks/components your web application is reliant upon and the vulnerabilities such components may be subject to.</t>
+          <t>['The web/application server is leaking information via one or more "X-Powered-By" HTTP response headers. Access to such information may facilitate attackers identifying other frameworks/components your web application is reliant upon and the vulnerabilities such components may be subject to.']</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ensure that your web server, application server, load balancer, etc. is configured to suppress "X-Powered-By" headers.</t>
+          <t>['Ensure that your web server, application server, load balancer, etc. is configured to suppress "X-Powered-By" headers.']</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -619,12 +618,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>The web/application server is leaking version information via the "Server" HTTP response header. Access to such information may facilitate attackers identifying other vulnerabilities your web/application server is subject to.</t>
+          <t>['The web/application server is leaking version information via the "Server" HTTP response header. Access to such information may facilitate attackers identifying other vulnerabilities your web/application server is subject to.']</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ensure that your web server, application server, load balancer, etc. is configured to suppress the "Server" header or provide generic details.</t>
+          <t>['Ensure that your web server, application server, load balancer, etc. is configured to suppress the "Server" header or provide generic details.']</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -663,13 +662,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>The Anti-MIME-Sniffing header X-Content-Type-Options was not set to 'nosniff'. This allows older versions of Internet Explorer and Chrome to perform MIME-sniffing on the response body, potentially causing the response body to be interpreted and displayed as a content type other than the declared content type. Current (early 2014) and legacy versions of Firefox will use the declared content type (if one is set), rather than performing MIME-sniffing.</t>
+          <t>["The Anti-MIME-Sniffing header X-Content-Type-Options was not set to 'nosniff'. This allows older versions of Internet Explorer and Chrome to perform MIME-sniffing on the response body, potentially causing the response body to be interpreted and displayed as a content type other than the declared content type. Current (early 2014) and legacy versions of Firefox will use the declared content type (if one is set), rather than performing MIME-sniffing."]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ensure that the application/web server sets the Content-Type header appropriately, and that it sets the X-Content-Type-Options header to 'nosniff' for all web pages.
-If possible, ensure that the end user uses a standards-compliant and modern web browser that does not perform MIME-sniffing at all, or that can be directed by the web application/web server to not perform MIME-sniffing.</t>
+          <t>["Ensure that the application/web server sets the Content-Type header appropriately, and that it sets the X-Content-Type-Options header to 'nosniff' for all web pages.", 'If possible, ensure that the end user uses a standards-compliant and modern web browser that does not perform MIME-sniffing at all, or that can be directed by the web application/web server to not perform MIME-sniffing.']</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -708,12 +706,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>The response appears to contain suspicious comments which may help an attacker.</t>
+          <t>['The response appears to contain suspicious comments which may help an attacker.']</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Remove all comments that return information that may help an attacker and fix any underlying problems they refer to.</t>
+          <t>['Remove all comments that return information that may help an attacker and fix any underlying problems they refer to.']</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -752,7 +750,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Check for differences in response based on fuzzed User Agent (eg. mobile sites, access as a Search Engine Crawler). Compares the response statuscode and the hashcode of the response body with the original response.</t>
+          <t>['Check for differences in response based on fuzzed User Agent (eg. mobile sites, access as a Search Engine Crawler). Compares the response statuscode and the hashcode of the response body with the original response.']</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>

</xml_diff>